<commit_message>
Cambios en como se entrenan los modelos
</commit_message>
<xml_diff>
--- a/Docs/MatricesConfusion.xlsx
+++ b/Docs/MatricesConfusion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabia\Desktop\Universidad\TesisML\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA18F641-AFCD-45C6-BF3A-E3BF930596F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7AFA10-C65E-4346-B271-A0D22AB11876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6AC4EB0C-B527-447A-9D72-F051D8CE6F27}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>Verdaderos Positivos = 0</t>
   </si>
@@ -74,7 +74,13 @@
     <t>Verdaderos Positivos = 36012</t>
   </si>
   <si>
-    <t>Falsos Negativos = 32613</t>
+    <t>Primera Prueba</t>
+  </si>
+  <si>
+    <t>Segunda Prueba</t>
+  </si>
+  <si>
+    <t>Falsos Positivos = 32613</t>
   </si>
 </sst>
 </file>
@@ -133,16 +139,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>18212</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>678180</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>140132</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>106679</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>487680</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>45719</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -172,7 +178,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4953000" y="383972"/>
+          <a:off x="8755380" y="140132"/>
           <a:ext cx="5356860" cy="3014547"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -512,38 +518,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DD31B2-5B19-4C15-9627-06AF987A52D0}">
-  <dimension ref="A2:C16"/>
+  <dimension ref="A2:G16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>0</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F3">
+        <v>7434</v>
+      </c>
+      <c r="G3">
+        <v>7910</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F4">
+        <v>22058</v>
+      </c>
+      <c r="G4">
+        <v>29306</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -551,23 +576,35 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>0</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F9">
+        <v>7704</v>
+      </c>
+      <c r="G9">
+        <v>8061</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>3</v>
       </c>
       <c r="C10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F10">
+        <v>21788</v>
+      </c>
+      <c r="G10">
+        <v>29155</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -575,20 +612,20 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>